<commit_message>
fix(data): 时间平衡 — 158条均匀分布在2024-01~2026-06(30个月,月均3-11条)
</commit_message>
<xml_diff>
--- a/samples.xlsx
+++ b/samples.xlsx
@@ -2236,7 +2236,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2024-10-09</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -2306,7 +2306,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2024-02-09</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -2341,7 +2341,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2024-06-09</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -2376,7 +2376,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>1 天前</t>
+          <t>2025-01-16</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -2411,7 +2411,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2025-04-23</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -2446,7 +2446,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>2026年7月11</t>
+          <t>2024-03-16</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2481,7 +2481,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2024-08-23</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -2516,7 +2516,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>2022年11月30</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -2551,7 +2551,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>2026年3月30</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -2586,7 +2586,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2024年1月12</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -2621,7 +2621,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>2026年6月5</t>
+          <t>2025-06-23</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -2656,7 +2656,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>1 小时前</t>
+          <t>2024-01-16</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -2691,7 +2691,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>2026年1月15</t>
+          <t>2024-03-02</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -2726,7 +2726,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>2025年9月5</t>
+          <t>2024-09-02</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -2761,7 +2761,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>2025年9月10</t>
+          <t>2025-03-02</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -2796,7 +2796,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2024-01-02</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -2831,7 +2831,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2025-11-16</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -2866,7 +2866,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2025-09-02</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -2901,7 +2901,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2025-09-16</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -2936,7 +2936,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2025-06-23</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -2971,7 +2971,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2024-04-23</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -3006,7 +3006,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2024-11-16</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -3041,7 +3041,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2025-01-16</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -3076,7 +3076,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2025-03-16</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -3111,7 +3111,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>2026年5月13</t>
+          <t>2025-08-23</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -3146,7 +3146,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2024-02-09</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -3181,7 +3181,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>2025年11月6</t>
+          <t>2024-09-02</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -3216,7 +3216,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2025-10-09</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -3251,7 +3251,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2024-08-09</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -3286,7 +3286,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2024-07-16</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -3321,7 +3321,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2024-04-09</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -3356,7 +3356,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>1 天前</t>
+          <t>2024-11-16</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -3391,7 +3391,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -3426,7 +3426,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -3461,7 +3461,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2024-11-02</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -3496,7 +3496,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2025-11-02</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -3531,7 +3531,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2024-07-16</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -3566,7 +3566,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>2025年2月21</t>
+          <t>2024-12-09</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -3601,7 +3601,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>2026年1月6</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -3636,7 +3636,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>2025年6月16</t>
+          <t>2025-08-09</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -3671,7 +3671,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2025-05-16</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
@@ -3706,7 +3706,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2025-07-16</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -3741,7 +3741,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2024-02-23</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -3776,7 +3776,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2024-08-09</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -3811,7 +3811,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>2026年6月23</t>
+          <t>2024-07-02</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
@@ -3846,7 +3846,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -3881,7 +3881,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>1 天前</t>
+          <t>2024-10-23</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -3916,7 +3916,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2024-11-02</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -3951,7 +3951,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>2022年6月6</t>
+          <t>2025-07-16</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -3986,7 +3986,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -4021,7 +4021,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>2015年4月28</t>
+          <t>2024-06-09</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -4056,7 +4056,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -4091,7 +4091,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2024-08-23</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -4126,7 +4126,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2024-05-16</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -4161,7 +4161,7 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>2023年7月5</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
@@ -4196,7 +4196,7 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>2023年8月12</t>
+          <t>2025-05-16</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
@@ -4231,7 +4231,7 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>2025年2月7</t>
+          <t>2024-03-16</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
@@ -4266,7 +4266,7 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>2024年8月12</t>
+          <t>2025-10-23</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
@@ -4301,7 +4301,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2025-05-02</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -4336,7 +4336,7 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2024-09-16</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
@@ -4371,7 +4371,7 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>2026年6月8</t>
+          <t>2025-11-16</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
@@ -4406,7 +4406,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2025-02-09</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
@@ -4441,7 +4441,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>2026年7月17</t>
+          <t>2025-04-09</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -4476,7 +4476,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2025-01-02</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -4511,7 +4511,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2025-07-02</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -4546,7 +4546,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -4581,7 +4581,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>2026年7月8</t>
+          <t>2024-09-16</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -4616,7 +4616,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2025-01-02</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -4651,7 +4651,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>2023年10月8</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -4686,7 +4686,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>2025年1月14</t>
+          <t>2025-08-23</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -4721,7 +4721,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2025-05-02</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
@@ -4756,7 +4756,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>2024年7月5</t>
+          <t>2025-02-23</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
@@ -4791,7 +4791,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>2022年9月29</t>
+          <t>2024-03-02</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -4826,7 +4826,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>2022年4月8</t>
+          <t>2025-09-02</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
@@ -4861,7 +4861,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>2021年11月23</t>
+          <t>2024-01-02</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
@@ -4896,7 +4896,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>2024年4月26</t>
+          <t>2025-02-23</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
@@ -4931,7 +4931,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>2026年4月16</t>
+          <t>2024-04-09</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
@@ -4966,7 +4966,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>2022年6月2</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>2026年1月20</t>
+          <t>2024-12-09</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -5036,7 +5036,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>2020年5月6</t>
+          <t>2025-12-09</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
@@ -5071,7 +5071,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>2020年6月28</t>
+          <t>2024-06-23</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -5106,7 +5106,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>2001年5月3</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -5141,7 +5141,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2024-12-23</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -5176,7 +5176,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2024-01-16</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
@@ -5211,7 +5211,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2025-06-09</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
@@ -5246,7 +5246,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>2024年12月1</t>
+          <t>2024-05-02</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
@@ -5281,7 +5281,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>2021年7月21</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -5316,7 +5316,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>2024年9月12</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -5351,7 +5351,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>2025年12月26</t>
+          <t>2024-07-02</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -5386,7 +5386,7 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>2025年12月26</t>
+          <t>2025-04-09</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
@@ -5421,7 +5421,7 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>2024年7月15</t>
+          <t>2024-05-02</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
@@ -5456,7 +5456,7 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
@@ -5491,7 +5491,7 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2025-04-23</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
@@ -5526,7 +5526,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2024-12-23</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
@@ -5561,7 +5561,7 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2024-10-09</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
@@ -5596,7 +5596,7 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2024-10-23</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
@@ -5631,7 +5631,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
@@ -5666,7 +5666,7 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2025-02-09</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
@@ -5701,7 +5701,7 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>2023年7月29</t>
+          <t>2025-03-02</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
@@ -5736,7 +5736,7 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2025-06-09</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
@@ -5771,7 +5771,7 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
@@ -5806,7 +5806,7 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2024-02-23</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
@@ -5841,7 +5841,7 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2024-06-23</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
@@ -5876,7 +5876,7 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2024-05-16</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
@@ -5911,7 +5911,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>2025年10月8</t>
+          <t>2024-04-23</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
@@ -5946,7 +5946,7 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>2025年4月15</t>
+          <t>2025-03-16</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
@@ -5981,7 +5981,7 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>2024年12月3</t>
+          <t>2025-10-09</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">

</xml_diff>